<commit_message>
pour publication 1.0.1 20cd66985a0d90bde5b54ce196171a9f67baff3a
</commit_message>
<xml_diff>
--- a/ig/publication-101/StructureDefinition-tddui-bundle.xlsx
+++ b/ig/publication-101/StructureDefinition-tddui-bundle.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.0.1-ballot</t>
+    <t>1.0.1</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-03-29T08:49:00+00:00</t>
+    <t>2024-03-29T09:04:17+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>